<commit_message>
주총일정 업데이트 (2026-03-15 23:51)
</commit_message>
<xml_diff>
--- a/주주총회.xlsx
+++ b/주주총회.xlsx
@@ -2020,10 +2020,8 @@
           <t>한미사이언스</t>
         </is>
       </c>
-      <c r="C73" s="44" t="inlineStr">
-        <is>
-          <t>미정 (25.3.26)</t>
-        </is>
+      <c r="C73" s="44" t="n">
+        <v>46112</v>
       </c>
       <c r="D73" s="45" t="n"/>
       <c r="E73" s="32" t="inlineStr">
@@ -2102,10 +2100,8 @@
           <t>한국금융지주</t>
         </is>
       </c>
-      <c r="C78" s="36" t="inlineStr">
-        <is>
-          <t>미정 (25.3.28)</t>
-        </is>
+      <c r="C78" s="36" t="n">
+        <v>46108</v>
       </c>
       <c r="D78" s="37" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
주총일정 업데이트 (2026-03-16 23:40)
</commit_message>
<xml_diff>
--- a/주주총회.xlsx
+++ b/주주총회.xlsx
@@ -2136,10 +2136,8 @@
           <t>글로벌텍스프리</t>
         </is>
       </c>
-      <c r="C80" s="44" t="inlineStr">
-        <is>
-          <t>미정 (25.3.31)</t>
-        </is>
+      <c r="C80" s="44" t="n">
+        <v>46112</v>
       </c>
       <c r="D80" s="45" t="n"/>
       <c r="E80" s="32" t="inlineStr">

</xml_diff>